<commit_message>
NEW FORMAT Balance: red when 0 as well as negative
Per sirichai: a zero Balance now also gets the red font (rule is
value <= 0, was < 0); positive stays blue. Re-built 2026-10-06.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/10-6/Stock Daily 2026-10-06.xlsx
+++ b/10-6/Stock Daily 2026-10-06.xlsx
@@ -22,7 +22,7 @@
     <numFmt numFmtId="165" formatCode="0;-0;;@"/>
     <numFmt numFmtId="166" formatCode="d/m/yyyy"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="27">
     <font>
       <name val="Tahoma"/>
       <family val="2"/>
@@ -183,6 +183,12 @@
       <color rgb="FF0000FF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="11">
     <fill>
@@ -1043,7 +1049,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="257">
+  <cellXfs count="258">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1770,6 +1776,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="13" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -7627,19 +7636,19 @@
         <f>SUM(G3+G4+G5+G6+G7-G8-G9)</f>
         <v/>
       </c>
-      <c r="H10" s="255">
+      <c r="H10" s="256">
         <f>SUM(H3+H4+H5+H6+H7-H8-H9)</f>
         <v/>
       </c>
-      <c r="I10" s="255">
+      <c r="I10" s="256">
         <f>SUM(I3+I4+I5+I6+I7-I8-I9)</f>
         <v/>
       </c>
-      <c r="J10" s="255">
+      <c r="J10" s="256">
         <f>SUM(J3+J4+J5+J6+J7-J8-J9)</f>
         <v/>
       </c>
-      <c r="K10" s="255">
+      <c r="K10" s="256">
         <f>SUM(K3+K4+K5+K6+K7-K8-K9)</f>
         <v/>
       </c>
@@ -7907,11 +7916,11 @@
         <f>Daily!AC41</f>
         <v/>
       </c>
-      <c r="I19" s="256">
+      <c r="I19" s="257">
         <f>Daily!AD41</f>
         <v/>
       </c>
-      <c r="J19" s="256">
+      <c r="J19" s="257">
         <f>Daily!AE41</f>
         <v/>
       </c>
@@ -7997,7 +8006,7 @@
         <f>SUM(G14+G15+G16+G17+G18-G19-G20)</f>
         <v/>
       </c>
-      <c r="H21" s="255">
+      <c r="H21" s="256">
         <f>SUM(H14+H15+H16+H17+H18-H19-H20)</f>
         <v/>
       </c>
@@ -8009,7 +8018,7 @@
         <f>SUM(J14+J15+J16+J17+J18-J19-J20)</f>
         <v/>
       </c>
-      <c r="K21" s="255">
+      <c r="K21" s="256">
         <f>SUM(K14+K15+K16+K17+K18-K19-K20)</f>
         <v/>
       </c>

</xml_diff>